<commit_message>
Add keyboard shortcuts for quiz traversal and update FAT questions
</commit_message>
<xml_diff>
--- a/FAT.xlsx
+++ b/FAT.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vrish\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vrish\Downloads\STS MCQS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{281AEC6B-1754-461E-A95A-82CE78A3BDAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45075142-5363-401C-8732-9E41914339F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{AA0512FE-C921-439A-A532-EE4DC374EB1D}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1951" uniqueCount="762">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1951" uniqueCount="763">
   <si>
     <t>Topic</t>
   </si>
@@ -1286,12 +1286,6 @@
     <t>What is the time complexity of LCS using Hirschberg's algorithm (divide and conquer)?</t>
   </si>
   <si>
-    <t>O(m*n) but O(min(m</t>
-  </si>
-  <si>
-    <t>n)) space</t>
-  </si>
-  <si>
     <t>LCS is not the same as:</t>
   </si>
   <si>
@@ -2322,6 +2316,15 @@
   </si>
   <si>
     <t>Uses less memory</t>
+  </si>
+  <si>
+    <t>O(max(m,n))</t>
+  </si>
+  <si>
+    <t>O(min(m,n))</t>
+  </si>
+  <si>
+    <t>O(m*n) but O(min(m,))</t>
   </si>
 </sst>
 </file>
@@ -2364,7 +2367,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -2387,11 +2390,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -2401,6 +2415,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5980,13 +5997,13 @@
         <v>377</v>
       </c>
       <c r="F125" s="2" t="s">
-        <v>380</v>
+        <v>760</v>
       </c>
       <c r="G125" s="2" t="s">
-        <v>381</v>
-      </c>
-      <c r="H125" s="2" t="s">
         <v>17</v>
+      </c>
+      <c r="H125" s="4" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="126" spans="1:8" ht="101.4" thickBot="1" x14ac:dyDescent="0.35">
@@ -6185,16 +6202,16 @@
         <v>376</v>
       </c>
       <c r="E133" s="2" t="s">
-        <v>408</v>
+        <v>761</v>
       </c>
       <c r="F133" s="2" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
       <c r="G133" s="2" t="s">
-        <v>377</v>
-      </c>
-      <c r="H133" s="2" t="s">
         <v>17</v>
+      </c>
+      <c r="H133" s="4" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="134" spans="1:8" ht="159" thickBot="1" x14ac:dyDescent="0.35">
@@ -6266,13 +6283,13 @@
         <v>376</v>
       </c>
       <c r="F136" s="2" t="s">
-        <v>416</v>
+        <v>762</v>
       </c>
       <c r="G136" s="2" t="s">
-        <v>417</v>
-      </c>
-      <c r="H136" s="2" t="s">
         <v>367</v>
+      </c>
+      <c r="H136" s="4" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="137" spans="1:8" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
@@ -6283,19 +6300,19 @@
         <v>51</v>
       </c>
       <c r="C137" s="3" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="D137" s="2" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="E137" s="2" t="s">
         <v>369</v>
       </c>
       <c r="F137" s="2" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="G137" s="2" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="H137" s="2" t="s">
         <v>21</v>
@@ -6309,19 +6326,19 @@
         <v>51</v>
       </c>
       <c r="C138" s="3" t="s">
+        <v>420</v>
+      </c>
+      <c r="D138" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="E138" s="2" t="s">
         <v>422</v>
       </c>
-      <c r="D138" s="2" t="s">
+      <c r="F138" s="2" t="s">
         <v>423</v>
       </c>
-      <c r="E138" s="2" t="s">
+      <c r="G138" s="2" t="s">
         <v>424</v>
-      </c>
-      <c r="F138" s="2" t="s">
-        <v>425</v>
-      </c>
-      <c r="G138" s="2" t="s">
-        <v>426</v>
       </c>
       <c r="H138" s="2" t="s">
         <v>21</v>
@@ -6335,7 +6352,7 @@
         <v>51</v>
       </c>
       <c r="C139" s="3" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="D139" s="2">
         <v>0</v>
@@ -6361,22 +6378,22 @@
         <v>51</v>
       </c>
       <c r="C140" s="3" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="D140" s="2" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="E140" s="2" t="s">
         <v>19</v>
       </c>
       <c r="F140" s="2" t="s">
-        <v>408</v>
+        <v>761</v>
       </c>
       <c r="G140" s="2" t="s">
-        <v>381</v>
-      </c>
-      <c r="H140" s="2" t="s">
         <v>377</v>
+      </c>
+      <c r="H140" s="4" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="141" spans="1:8" ht="130.19999999999999" thickBot="1" x14ac:dyDescent="0.35">
@@ -6387,19 +6404,19 @@
         <v>51</v>
       </c>
       <c r="C141" s="3" t="s">
+        <v>428</v>
+      </c>
+      <c r="D141" s="2" t="s">
+        <v>429</v>
+      </c>
+      <c r="E141" s="2" t="s">
         <v>430</v>
       </c>
-      <c r="D141" s="2" t="s">
+      <c r="F141" s="2" t="s">
         <v>431</v>
       </c>
-      <c r="E141" s="2" t="s">
+      <c r="G141" s="2" t="s">
         <v>432</v>
-      </c>
-      <c r="F141" s="2" t="s">
-        <v>433</v>
-      </c>
-      <c r="G141" s="2" t="s">
-        <v>434</v>
       </c>
       <c r="H141" s="2" t="s">
         <v>15</v>
@@ -6413,7 +6430,7 @@
         <v>88</v>
       </c>
       <c r="C142" s="3" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="D142" s="2" t="s">
         <v>20</v>
@@ -6439,7 +6456,7 @@
         <v>88</v>
       </c>
       <c r="C143" s="3" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="D143" s="2" t="s">
         <v>19</v>
@@ -6465,19 +6482,19 @@
         <v>88</v>
       </c>
       <c r="C144" s="3" t="s">
+        <v>435</v>
+      </c>
+      <c r="D144" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="E144" s="2" t="s">
         <v>437</v>
       </c>
-      <c r="D144" s="2" t="s">
+      <c r="F144" s="2" t="s">
         <v>438</v>
       </c>
-      <c r="E144" s="2" t="s">
+      <c r="G144" s="2" t="s">
         <v>439</v>
-      </c>
-      <c r="F144" s="2" t="s">
-        <v>440</v>
-      </c>
-      <c r="G144" s="2" t="s">
-        <v>441</v>
       </c>
       <c r="H144" s="2" t="s">
         <v>21</v>
@@ -6491,19 +6508,19 @@
         <v>88</v>
       </c>
       <c r="C145" s="3" t="s">
+        <v>440</v>
+      </c>
+      <c r="D145" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="E145" s="2" t="s">
         <v>442</v>
       </c>
-      <c r="D145" s="2" t="s">
+      <c r="F145" s="2" t="s">
         <v>443</v>
       </c>
-      <c r="E145" s="2" t="s">
+      <c r="G145" s="2" t="s">
         <v>444</v>
-      </c>
-      <c r="F145" s="2" t="s">
-        <v>445</v>
-      </c>
-      <c r="G145" s="2" t="s">
-        <v>446</v>
       </c>
       <c r="H145" s="2" t="s">
         <v>21</v>
@@ -6517,7 +6534,7 @@
         <v>88</v>
       </c>
       <c r="C146" s="3" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="D146" s="2" t="s">
         <v>63</v>
@@ -6529,7 +6546,7 @@
         <v>62</v>
       </c>
       <c r="G146" s="2" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="H146" s="2" t="s">
         <v>21</v>
@@ -6543,7 +6560,7 @@
         <v>88</v>
       </c>
       <c r="C147" s="3" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="D147" s="2">
         <v>10</v>
@@ -6569,19 +6586,19 @@
         <v>88</v>
       </c>
       <c r="C148" s="3" t="s">
+        <v>448</v>
+      </c>
+      <c r="D148" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="E148" s="2" t="s">
         <v>450</v>
       </c>
-      <c r="D148" s="2" t="s">
+      <c r="F148" s="2" t="s">
         <v>451</v>
       </c>
-      <c r="E148" s="2" t="s">
+      <c r="G148" s="2" t="s">
         <v>452</v>
-      </c>
-      <c r="F148" s="2" t="s">
-        <v>453</v>
-      </c>
-      <c r="G148" s="2" t="s">
-        <v>454</v>
       </c>
       <c r="H148" s="2" t="s">
         <v>21</v>
@@ -6595,10 +6612,10 @@
         <v>88</v>
       </c>
       <c r="C149" s="3" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="D149" s="2" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="E149" s="2" t="s">
         <v>413</v>
@@ -6607,7 +6624,7 @@
         <v>278</v>
       </c>
       <c r="G149" s="2" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="H149" s="2" t="s">
         <v>21</v>
@@ -6621,7 +6638,7 @@
         <v>88</v>
       </c>
       <c r="C150" s="3" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="D150" s="2" t="s">
         <v>408</v>
@@ -6647,16 +6664,16 @@
         <v>88</v>
       </c>
       <c r="C151" s="3" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="D151" s="2" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="E151" s="2" t="s">
         <v>377</v>
       </c>
       <c r="F151" s="2" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="G151" s="2" t="s">
         <v>54</v>
@@ -6667,13 +6684,13 @@
     </row>
     <row r="152" spans="1:8" ht="87" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A152" s="2" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B152" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C152" s="3" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="D152" s="2">
         <v>2</v>
@@ -6693,13 +6710,13 @@
     </row>
     <row r="153" spans="1:8" ht="115.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A153" s="2" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B153" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C153" s="3" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="D153" s="2" t="s">
         <v>19</v>
@@ -6719,13 +6736,13 @@
     </row>
     <row r="154" spans="1:8" ht="101.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A154" s="2" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B154" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C154" s="3" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="D154" s="2" t="s">
         <v>17</v>
@@ -6745,25 +6762,25 @@
     </row>
     <row r="155" spans="1:8" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A155" s="2" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B155" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C155" s="3" t="s">
+        <v>464</v>
+      </c>
+      <c r="D155" s="2" t="s">
+        <v>465</v>
+      </c>
+      <c r="E155" s="2" t="s">
         <v>466</v>
       </c>
-      <c r="D155" s="2" t="s">
+      <c r="F155" s="2" t="s">
+        <v>455</v>
+      </c>
+      <c r="G155" s="2" t="s">
         <v>467</v>
-      </c>
-      <c r="E155" s="2" t="s">
-        <v>468</v>
-      </c>
-      <c r="F155" s="2" t="s">
-        <v>457</v>
-      </c>
-      <c r="G155" s="2" t="s">
-        <v>469</v>
       </c>
       <c r="H155" s="2" t="s">
         <v>21</v>
@@ -6771,13 +6788,13 @@
     </row>
     <row r="156" spans="1:8" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A156" s="2" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B156" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C156" s="3" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="D156" s="2">
         <v>1</v>
@@ -6797,13 +6814,13 @@
     </row>
     <row r="157" spans="1:8" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A157" s="2" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B157" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C157" s="3" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="D157" s="2">
         <v>1</v>
@@ -6823,25 +6840,25 @@
     </row>
     <row r="158" spans="1:8" ht="130.19999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A158" s="2" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B158" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C158" s="3" t="s">
+        <v>470</v>
+      </c>
+      <c r="D158" s="2" t="s">
+        <v>471</v>
+      </c>
+      <c r="E158" s="2" t="s">
         <v>472</v>
       </c>
-      <c r="D158" s="2" t="s">
+      <c r="F158" s="2" t="s">
         <v>473</v>
       </c>
-      <c r="E158" s="2" t="s">
+      <c r="G158" s="2" t="s">
         <v>474</v>
-      </c>
-      <c r="F158" s="2" t="s">
-        <v>475</v>
-      </c>
-      <c r="G158" s="2" t="s">
-        <v>476</v>
       </c>
       <c r="H158" s="2" t="s">
         <v>21</v>
@@ -6849,13 +6866,13 @@
     </row>
     <row r="159" spans="1:8" ht="144.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A159" s="2" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B159" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C159" s="3" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="D159" s="2" t="s">
         <v>19</v>
@@ -6875,13 +6892,13 @@
     </row>
     <row r="160" spans="1:8" ht="101.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A160" s="2" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B160" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C160" s="3" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="D160" s="2">
         <v>1</v>
@@ -6901,25 +6918,25 @@
     </row>
     <row r="161" spans="1:8" ht="101.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A161" s="2" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B161" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C161" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="D161" s="2" t="s">
+        <v>478</v>
+      </c>
+      <c r="E161" s="2" t="s">
         <v>479</v>
       </c>
-      <c r="D161" s="2" t="s">
+      <c r="F161" s="2" t="s">
         <v>480</v>
       </c>
-      <c r="E161" s="2" t="s">
+      <c r="G161" s="2" t="s">
         <v>481</v>
-      </c>
-      <c r="F161" s="2" t="s">
-        <v>482</v>
-      </c>
-      <c r="G161" s="2" t="s">
-        <v>483</v>
       </c>
       <c r="H161" s="2" t="s">
         <v>21</v>
@@ -6927,13 +6944,13 @@
     </row>
     <row r="162" spans="1:8" ht="115.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A162" s="2" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B162" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C162" s="3" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="D162" s="2">
         <v>4</v>
@@ -6953,25 +6970,25 @@
     </row>
     <row r="163" spans="1:8" ht="130.19999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A163" s="2" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B163" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C163" s="3" t="s">
+        <v>483</v>
+      </c>
+      <c r="D163" s="2" t="s">
+        <v>484</v>
+      </c>
+      <c r="E163" s="2" t="s">
+        <v>467</v>
+      </c>
+      <c r="F163" s="2" t="s">
         <v>485</v>
       </c>
-      <c r="D163" s="2" t="s">
+      <c r="G163" s="2" t="s">
         <v>486</v>
-      </c>
-      <c r="E163" s="2" t="s">
-        <v>469</v>
-      </c>
-      <c r="F163" s="2" t="s">
-        <v>487</v>
-      </c>
-      <c r="G163" s="2" t="s">
-        <v>488</v>
       </c>
       <c r="H163" s="2" t="s">
         <v>29</v>
@@ -6979,13 +6996,13 @@
     </row>
     <row r="164" spans="1:8" ht="115.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A164" s="2" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B164" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C164" s="3" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="D164" s="2" t="s">
         <v>17</v>
@@ -7005,13 +7022,13 @@
     </row>
     <row r="165" spans="1:8" ht="144.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A165" s="2" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B165" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C165" s="3" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="D165" s="2" t="s">
         <v>19</v>
@@ -7031,13 +7048,13 @@
     </row>
     <row r="166" spans="1:8" ht="202.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A166" s="2" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B166" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C166" s="3" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="D166" s="2" t="s">
         <v>19</v>
@@ -7057,13 +7074,13 @@
     </row>
     <row r="167" spans="1:8" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A167" s="2" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B167" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C167" s="3" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="D167" s="2">
         <v>3</v>
@@ -7083,22 +7100,22 @@
     </row>
     <row r="168" spans="1:8" ht="115.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A168" s="2" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B168" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C168" s="3" t="s">
+        <v>491</v>
+      </c>
+      <c r="D168" s="2" t="s">
+        <v>492</v>
+      </c>
+      <c r="E168" s="2" t="s">
         <v>493</v>
       </c>
-      <c r="D168" s="2" t="s">
+      <c r="F168" s="2" t="s">
         <v>494</v>
-      </c>
-      <c r="E168" s="2" t="s">
-        <v>495</v>
-      </c>
-      <c r="F168" s="2" t="s">
-        <v>496</v>
       </c>
       <c r="G168" s="2" t="s">
         <v>149</v>
@@ -7109,22 +7126,22 @@
     </row>
     <row r="169" spans="1:8" ht="115.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A169" s="2" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B169" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C169" s="3" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
       <c r="D169" s="2" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="E169" s="2" t="s">
         <v>247</v>
       </c>
       <c r="F169" s="2" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="G169" s="2" t="s">
         <v>351</v>
@@ -7135,13 +7152,13 @@
     </row>
     <row r="170" spans="1:8" ht="101.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A170" s="2" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B170" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C170" s="3" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="D170" s="2" t="s">
         <v>20</v>
@@ -7161,25 +7178,25 @@
     </row>
     <row r="171" spans="1:8" ht="115.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A171" s="2" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B171" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C171" s="3" t="s">
+        <v>499</v>
+      </c>
+      <c r="D171" s="2" t="s">
+        <v>500</v>
+      </c>
+      <c r="E171" s="2" t="s">
         <v>501</v>
-      </c>
-      <c r="D171" s="2" t="s">
-        <v>502</v>
-      </c>
-      <c r="E171" s="2" t="s">
-        <v>503</v>
       </c>
       <c r="F171" s="2" t="s">
         <v>33</v>
       </c>
       <c r="G171" s="2" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="H171" s="2" t="s">
         <v>21</v>
@@ -7187,13 +7204,13 @@
     </row>
     <row r="172" spans="1:8" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A172" s="2" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B172" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C172" s="3" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="D172" s="2">
         <v>5</v>
@@ -7213,25 +7230,25 @@
     </row>
     <row r="173" spans="1:8" ht="187.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A173" s="2" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B173" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C173" s="3" t="s">
+        <v>504</v>
+      </c>
+      <c r="D173" s="2" t="s">
+        <v>505</v>
+      </c>
+      <c r="E173" s="2" t="s">
         <v>506</v>
       </c>
-      <c r="D173" s="2" t="s">
+      <c r="F173" s="2" t="s">
         <v>507</v>
       </c>
-      <c r="E173" s="2" t="s">
+      <c r="G173" s="2" t="s">
         <v>508</v>
-      </c>
-      <c r="F173" s="2" t="s">
-        <v>509</v>
-      </c>
-      <c r="G173" s="2" t="s">
-        <v>510</v>
       </c>
       <c r="H173" s="2" t="s">
         <v>21</v>
@@ -7239,13 +7256,13 @@
     </row>
     <row r="174" spans="1:8" ht="173.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A174" s="2" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B174" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C174" s="3" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="D174" s="2" t="s">
         <v>54</v>
@@ -7265,25 +7282,25 @@
     </row>
     <row r="175" spans="1:8" ht="144.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A175" s="2" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B175" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C175" s="3" t="s">
+        <v>510</v>
+      </c>
+      <c r="D175" s="2" t="s">
+        <v>511</v>
+      </c>
+      <c r="E175" s="2" t="s">
         <v>512</v>
       </c>
-      <c r="D175" s="2" t="s">
+      <c r="F175" s="2" t="s">
         <v>513</v>
       </c>
-      <c r="E175" s="2" t="s">
+      <c r="G175" s="2" t="s">
         <v>514</v>
-      </c>
-      <c r="F175" s="2" t="s">
-        <v>515</v>
-      </c>
-      <c r="G175" s="2" t="s">
-        <v>516</v>
       </c>
       <c r="H175" s="2" t="s">
         <v>21</v>
@@ -7291,16 +7308,16 @@
     </row>
     <row r="176" spans="1:8" ht="159" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A176" s="2" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B176" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C176" s="3" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="D176" s="2" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="E176" s="2" t="s">
         <v>213</v>
@@ -7317,25 +7334,25 @@
     </row>
     <row r="177" spans="1:8" ht="216.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A177" s="2" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B177" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C177" s="3" t="s">
+        <v>517</v>
+      </c>
+      <c r="D177" s="2" t="s">
+        <v>518</v>
+      </c>
+      <c r="E177" s="2" t="s">
         <v>519</v>
       </c>
-      <c r="D177" s="2" t="s">
+      <c r="F177" s="2" t="s">
         <v>520</v>
       </c>
-      <c r="E177" s="2" t="s">
+      <c r="G177" s="2" t="s">
         <v>521</v>
-      </c>
-      <c r="F177" s="2" t="s">
-        <v>522</v>
-      </c>
-      <c r="G177" s="2" t="s">
-        <v>523</v>
       </c>
       <c r="H177" s="2" t="s">
         <v>21</v>
@@ -7343,25 +7360,25 @@
     </row>
     <row r="178" spans="1:8" ht="144.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A178" s="2" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B178" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C178" s="3" t="s">
+        <v>522</v>
+      </c>
+      <c r="D178" s="2" t="s">
+        <v>523</v>
+      </c>
+      <c r="E178" s="2" t="s">
         <v>524</v>
       </c>
-      <c r="D178" s="2" t="s">
+      <c r="F178" s="2" t="s">
         <v>525</v>
       </c>
-      <c r="E178" s="2" t="s">
+      <c r="G178" s="2" t="s">
         <v>526</v>
-      </c>
-      <c r="F178" s="2" t="s">
-        <v>527</v>
-      </c>
-      <c r="G178" s="2" t="s">
-        <v>528</v>
       </c>
       <c r="H178" s="2" t="s">
         <v>21</v>
@@ -7369,13 +7386,13 @@
     </row>
     <row r="179" spans="1:8" ht="202.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A179" s="2" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B179" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C179" s="3" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="D179" s="2" t="s">
         <v>20</v>
@@ -7384,7 +7401,7 @@
         <v>54</v>
       </c>
       <c r="F179" s="2" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="G179" s="2" t="s">
         <v>19</v>
@@ -7395,25 +7412,25 @@
     </row>
     <row r="180" spans="1:8" ht="159" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A180" s="2" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B180" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C180" s="3" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="D180" s="2" t="s">
+        <v>511</v>
+      </c>
+      <c r="E180" s="2" t="s">
+        <v>512</v>
+      </c>
+      <c r="F180" s="2" t="s">
         <v>513</v>
       </c>
-      <c r="E180" s="2" t="s">
-        <v>514</v>
-      </c>
-      <c r="F180" s="2" t="s">
-        <v>515</v>
-      </c>
       <c r="G180" s="2" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="H180" s="2" t="s">
         <v>21</v>
@@ -7421,13 +7438,13 @@
     </row>
     <row r="181" spans="1:8" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A181" s="2" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B181" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C181" s="3" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="D181" s="2">
         <v>5</v>
@@ -7447,25 +7464,25 @@
     </row>
     <row r="182" spans="1:8" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A182" s="2" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="B182" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C182" s="3" t="s">
+        <v>533</v>
+      </c>
+      <c r="D182" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="E182" s="2" t="s">
         <v>535</v>
       </c>
-      <c r="D182" s="2" t="s">
+      <c r="F182" s="2" t="s">
         <v>536</v>
       </c>
-      <c r="E182" s="2" t="s">
+      <c r="G182" s="2" t="s">
         <v>537</v>
-      </c>
-      <c r="F182" s="2" t="s">
-        <v>538</v>
-      </c>
-      <c r="G182" s="2" t="s">
-        <v>539</v>
       </c>
       <c r="H182" s="2" t="s">
         <v>21</v>
@@ -7473,13 +7490,13 @@
     </row>
     <row r="183" spans="1:8" ht="130.19999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A183" s="2" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="B183" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C183" s="3" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="D183" s="2" t="s">
         <v>19</v>
@@ -7488,7 +7505,7 @@
         <v>54</v>
       </c>
       <c r="F183" s="2" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
       <c r="G183" s="2" t="s">
         <v>298</v>
@@ -7499,13 +7516,13 @@
     </row>
     <row r="184" spans="1:8" ht="101.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A184" s="2" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="B184" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C184" s="3" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
       <c r="D184" s="2" t="s">
         <v>19</v>
@@ -7525,13 +7542,13 @@
     </row>
     <row r="185" spans="1:8" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A185" s="2" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="B185" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C185" s="3" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="D185" s="2">
         <v>1</v>
@@ -7551,13 +7568,13 @@
     </row>
     <row r="186" spans="1:8" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A186" s="2" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="B186" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C186" s="3" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="D186" s="2">
         <v>0</v>
@@ -7577,25 +7594,25 @@
     </row>
     <row r="187" spans="1:8" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A187" s="2" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="B187" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C187" s="3" t="s">
+        <v>543</v>
+      </c>
+      <c r="D187" s="2" t="s">
+        <v>544</v>
+      </c>
+      <c r="E187" s="2" t="s">
         <v>545</v>
       </c>
-      <c r="D187" s="2" t="s">
+      <c r="F187" s="2" t="s">
         <v>546</v>
       </c>
-      <c r="E187" s="2" t="s">
+      <c r="G187" s="2" t="s">
         <v>547</v>
-      </c>
-      <c r="F187" s="2" t="s">
-        <v>548</v>
-      </c>
-      <c r="G187" s="2" t="s">
-        <v>549</v>
       </c>
       <c r="H187" s="2" t="s">
         <v>21</v>
@@ -7603,13 +7620,13 @@
     </row>
     <row r="188" spans="1:8" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A188" s="2" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="B188" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C188" s="3" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="D188" s="2">
         <v>2</v>
@@ -7629,13 +7646,13 @@
     </row>
     <row r="189" spans="1:8" ht="87" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A189" s="2" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="B189" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C189" s="3" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="D189" s="2" t="s">
         <v>226</v>
@@ -7655,13 +7672,13 @@
     </row>
     <row r="190" spans="1:8" ht="87" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A190" s="2" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="B190" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C190" s="3" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
       <c r="D190" s="2">
         <v>0</v>
@@ -7681,13 +7698,13 @@
     </row>
     <row r="191" spans="1:8" ht="87" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A191" s="2" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="B191" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C191" s="3" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="D191" s="2">
         <v>5</v>
@@ -7707,13 +7724,13 @@
     </row>
     <row r="192" spans="1:8" ht="101.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A192" s="2" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="B192" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C192" s="3" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="D192" s="2" t="s">
         <v>19</v>
@@ -7733,13 +7750,13 @@
     </row>
     <row r="193" spans="1:8" ht="144.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A193" s="2" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="B193" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C193" s="3" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
       <c r="D193" s="2">
         <v>1000000</v>
@@ -7759,19 +7776,19 @@
     </row>
     <row r="194" spans="1:8" ht="87" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A194" s="2" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="B194" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C194" s="3" t="s">
+        <v>554</v>
+      </c>
+      <c r="D194" s="2" t="s">
+        <v>555</v>
+      </c>
+      <c r="E194" s="2" t="s">
         <v>556</v>
-      </c>
-      <c r="D194" s="2" t="s">
-        <v>557</v>
-      </c>
-      <c r="E194" s="2" t="s">
-        <v>558</v>
       </c>
       <c r="F194" s="2">
         <v>1</v>
@@ -7785,22 +7802,22 @@
     </row>
     <row r="195" spans="1:8" ht="87" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A195" s="2" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="B195" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C195" s="3" t="s">
+        <v>557</v>
+      </c>
+      <c r="D195" s="2" t="s">
+        <v>558</v>
+      </c>
+      <c r="E195" s="2" t="s">
         <v>559</v>
       </c>
-      <c r="D195" s="2" t="s">
+      <c r="F195" s="2" t="s">
         <v>560</v>
-      </c>
-      <c r="E195" s="2" t="s">
-        <v>561</v>
-      </c>
-      <c r="F195" s="2" t="s">
-        <v>562</v>
       </c>
       <c r="G195" s="2" t="s">
         <v>396</v>
@@ -7811,22 +7828,22 @@
     </row>
     <row r="196" spans="1:8" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A196" s="2" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="B196" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C196" s="3" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="D196" s="2" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="E196" s="2" t="s">
+        <v>560</v>
+      </c>
+      <c r="F196" s="2" t="s">
         <v>562</v>
-      </c>
-      <c r="F196" s="2" t="s">
-        <v>564</v>
       </c>
       <c r="G196" s="2" t="s">
         <v>396</v>
@@ -7837,13 +7854,13 @@
     </row>
     <row r="197" spans="1:8" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A197" s="2" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="B197" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C197" s="3" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="D197" s="2">
         <v>3</v>
@@ -7863,13 +7880,13 @@
     </row>
     <row r="198" spans="1:8" ht="115.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A198" s="2" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="B198" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C198" s="3" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
       <c r="D198" s="2" t="s">
         <v>54</v>
@@ -7889,13 +7906,13 @@
     </row>
     <row r="199" spans="1:8" ht="115.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A199" s="2" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="B199" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C199" s="3" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="D199" s="2" t="s">
         <v>54</v>
@@ -7915,13 +7932,13 @@
     </row>
     <row r="200" spans="1:8" ht="101.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A200" s="2" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="B200" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C200" s="3" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
       <c r="D200" s="2">
         <v>10</v>
@@ -7941,25 +7958,25 @@
     </row>
     <row r="201" spans="1:8" ht="87" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A201" s="2" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="B201" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C201" s="3" t="s">
+        <v>567</v>
+      </c>
+      <c r="D201" s="2" t="s">
+        <v>568</v>
+      </c>
+      <c r="E201" s="2" t="s">
         <v>569</v>
       </c>
-      <c r="D201" s="2" t="s">
+      <c r="F201" s="2" t="s">
         <v>570</v>
       </c>
-      <c r="E201" s="2" t="s">
+      <c r="G201" s="2" t="s">
         <v>571</v>
-      </c>
-      <c r="F201" s="2" t="s">
-        <v>572</v>
-      </c>
-      <c r="G201" s="2" t="s">
-        <v>573</v>
       </c>
       <c r="H201" s="2" t="s">
         <v>21</v>
@@ -7967,13 +7984,13 @@
     </row>
     <row r="202" spans="1:8" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A202" s="2" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="B202" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C202" s="3" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="D202" s="2">
         <v>4</v>
@@ -7993,13 +8010,13 @@
     </row>
     <row r="203" spans="1:8" ht="173.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A203" s="2" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="B203" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C203" s="3" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="D203" s="2" t="s">
         <v>19</v>
@@ -8011,7 +8028,7 @@
         <v>54</v>
       </c>
       <c r="G203" s="2" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="H203" s="2" t="s">
         <v>23</v>
@@ -8019,25 +8036,25 @@
     </row>
     <row r="204" spans="1:8" ht="159" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A204" s="2" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="B204" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C204" s="3" t="s">
+        <v>575</v>
+      </c>
+      <c r="D204" s="2" t="s">
+        <v>576</v>
+      </c>
+      <c r="E204" s="2" t="s">
         <v>577</v>
       </c>
-      <c r="D204" s="2" t="s">
-        <v>578</v>
-      </c>
-      <c r="E204" s="2" t="s">
-        <v>579</v>
-      </c>
       <c r="F204" s="2" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="G204" s="2" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="H204" s="2" t="s">
         <v>21</v>
@@ -8045,13 +8062,13 @@
     </row>
     <row r="205" spans="1:8" ht="130.19999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A205" s="2" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="B205" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C205" s="3" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="D205" s="2" t="s">
         <v>19</v>
@@ -8071,13 +8088,13 @@
     </row>
     <row r="206" spans="1:8" ht="231" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A206" s="2" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="B206" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C206" s="3" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="D206" s="2" t="s">
         <v>19</v>
@@ -8089,7 +8106,7 @@
         <v>54</v>
       </c>
       <c r="G206" s="2" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="H206" s="2" t="s">
         <v>23</v>
@@ -8097,13 +8114,13 @@
     </row>
     <row r="207" spans="1:8" ht="101.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A207" s="2" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="B207" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C207" s="3" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="D207" s="2">
         <v>1</v>
@@ -8112,10 +8129,10 @@
         <v>2</v>
       </c>
       <c r="F207" s="2" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="G207" s="2" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="H207" s="2" t="s">
         <v>21</v>
@@ -8123,25 +8140,25 @@
     </row>
     <row r="208" spans="1:8" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A208" s="2" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="B208" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C208" s="3" t="s">
+        <v>581</v>
+      </c>
+      <c r="D208" s="2" t="s">
+        <v>582</v>
+      </c>
+      <c r="E208" s="2" t="s">
         <v>583</v>
       </c>
-      <c r="D208" s="2" t="s">
+      <c r="F208" s="2" t="s">
         <v>584</v>
       </c>
-      <c r="E208" s="2" t="s">
+      <c r="G208" s="2" t="s">
         <v>585</v>
-      </c>
-      <c r="F208" s="2" t="s">
-        <v>586</v>
-      </c>
-      <c r="G208" s="2" t="s">
-        <v>587</v>
       </c>
       <c r="H208" s="2" t="s">
         <v>21</v>
@@ -8149,16 +8166,16 @@
     </row>
     <row r="209" spans="1:8" ht="87" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A209" s="2" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="B209" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C209" s="3" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="D209" s="2" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="E209" s="2" t="s">
         <v>278</v>
@@ -8167,7 +8184,7 @@
         <v>413</v>
       </c>
       <c r="G209" s="2" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="H209" s="2" t="s">
         <v>21</v>
@@ -8175,13 +8192,13 @@
     </row>
     <row r="210" spans="1:8" ht="130.19999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A210" s="2" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="B210" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C210" s="3" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="D210" s="2" t="s">
         <v>298</v>
@@ -8201,13 +8218,13 @@
     </row>
     <row r="211" spans="1:8" ht="231" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A211" s="2" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="B211" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C211" s="3" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="D211" s="2" t="s">
         <v>19</v>
@@ -8227,25 +8244,25 @@
     </row>
     <row r="212" spans="1:8" ht="159" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A212" s="2" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="B212" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C212" s="3" t="s">
+        <v>592</v>
+      </c>
+      <c r="D212" s="2" t="s">
+        <v>593</v>
+      </c>
+      <c r="E212" s="2" t="s">
         <v>594</v>
       </c>
-      <c r="D212" s="2" t="s">
+      <c r="F212" s="2" t="s">
         <v>595</v>
       </c>
-      <c r="E212" s="2" t="s">
+      <c r="G212" s="2" t="s">
         <v>596</v>
-      </c>
-      <c r="F212" s="2" t="s">
-        <v>597</v>
-      </c>
-      <c r="G212" s="2" t="s">
-        <v>598</v>
       </c>
       <c r="H212" s="2" t="s">
         <v>21</v>
@@ -8253,25 +8270,25 @@
     </row>
     <row r="213" spans="1:8" ht="202.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A213" s="2" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="B213" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C213" s="3" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
       <c r="D213" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E213" s="2" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="F213" s="2" t="s">
         <v>298</v>
       </c>
       <c r="G213" s="2" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="H213" s="2" t="s">
         <v>23</v>
@@ -8279,25 +8296,25 @@
     </row>
     <row r="214" spans="1:8" ht="130.19999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A214" s="2" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="B214" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C214" s="3" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="D214" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E214" s="2" t="s">
+        <v>599</v>
+      </c>
+      <c r="F214" s="2" t="s">
+        <v>598</v>
+      </c>
+      <c r="G214" s="2" t="s">
         <v>601</v>
-      </c>
-      <c r="F214" s="2" t="s">
-        <v>600</v>
-      </c>
-      <c r="G214" s="2" t="s">
-        <v>603</v>
       </c>
       <c r="H214" s="2" t="s">
         <v>29</v>
@@ -8305,25 +8322,25 @@
     </row>
     <row r="215" spans="1:8" ht="101.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A215" s="2" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="B215" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C215" s="3" t="s">
+        <v>602</v>
+      </c>
+      <c r="D215" s="2" t="s">
+        <v>603</v>
+      </c>
+      <c r="E215" s="2" t="s">
         <v>604</v>
       </c>
-      <c r="D215" s="2" t="s">
+      <c r="F215" s="2" t="s">
         <v>605</v>
       </c>
-      <c r="E215" s="2" t="s">
-        <v>606</v>
-      </c>
-      <c r="F215" s="2" t="s">
-        <v>607</v>
-      </c>
       <c r="G215" s="2" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="H215" s="2" t="s">
         <v>21</v>
@@ -8331,25 +8348,25 @@
     </row>
     <row r="216" spans="1:8" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A216" s="2" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="B216" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C216" s="3" t="s">
+        <v>606</v>
+      </c>
+      <c r="D216" s="2" t="s">
+        <v>607</v>
+      </c>
+      <c r="E216" s="2" t="s">
         <v>608</v>
       </c>
-      <c r="D216" s="2" t="s">
+      <c r="F216" s="2" t="s">
         <v>609</v>
       </c>
-      <c r="E216" s="2" t="s">
+      <c r="G216" s="2" t="s">
         <v>610</v>
-      </c>
-      <c r="F216" s="2" t="s">
-        <v>611</v>
-      </c>
-      <c r="G216" s="2" t="s">
-        <v>612</v>
       </c>
       <c r="H216" s="2" t="s">
         <v>21</v>
@@ -8357,13 +8374,13 @@
     </row>
     <row r="217" spans="1:8" ht="130.19999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A217" s="2" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="B217" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C217" s="3" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="D217" s="2" t="s">
         <v>278</v>
@@ -8383,22 +8400,22 @@
     </row>
     <row r="218" spans="1:8" ht="187.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A218" s="2" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="B218" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C218" s="3" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="D218" s="2" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="E218" s="2" t="s">
         <v>227</v>
       </c>
       <c r="F218" s="2" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="G218" s="2" t="s">
         <v>278</v>
@@ -8409,25 +8426,25 @@
     </row>
     <row r="219" spans="1:8" ht="87" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A219" s="2" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="B219" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C219" s="3" t="s">
+        <v>615</v>
+      </c>
+      <c r="D219" s="2" t="s">
+        <v>616</v>
+      </c>
+      <c r="E219" s="2" t="s">
+        <v>604</v>
+      </c>
+      <c r="F219" s="2" t="s">
         <v>617</v>
       </c>
-      <c r="D219" s="2" t="s">
-        <v>618</v>
-      </c>
-      <c r="E219" s="2" t="s">
-        <v>606</v>
-      </c>
-      <c r="F219" s="2" t="s">
-        <v>619</v>
-      </c>
       <c r="G219" s="2" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="H219" s="2" t="s">
         <v>21</v>
@@ -8435,13 +8452,13 @@
     </row>
     <row r="220" spans="1:8" ht="115.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A220" s="2" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="B220" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C220" s="3" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="D220" s="2" t="b">
         <v>1</v>
@@ -8450,7 +8467,7 @@
         <v>0</v>
       </c>
       <c r="F220" s="2" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="G220" s="2" t="s">
         <v>87</v>
@@ -8461,22 +8478,22 @@
     </row>
     <row r="221" spans="1:8" ht="101.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A221" s="2" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="B221" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C221" s="3" t="s">
+        <v>620</v>
+      </c>
+      <c r="D221" s="2" t="s">
+        <v>621</v>
+      </c>
+      <c r="E221" s="2" t="s">
         <v>622</v>
       </c>
-      <c r="D221" s="2" t="s">
+      <c r="F221" s="2" t="s">
         <v>623</v>
-      </c>
-      <c r="E221" s="2" t="s">
-        <v>624</v>
-      </c>
-      <c r="F221" s="2" t="s">
-        <v>625</v>
       </c>
       <c r="G221" s="2" t="s">
         <v>149</v>
@@ -8487,25 +8504,25 @@
     </row>
     <row r="222" spans="1:8" ht="144.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A222" s="2" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="B222" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C222" s="3" t="s">
+        <v>624</v>
+      </c>
+      <c r="D222" s="2" t="s">
+        <v>625</v>
+      </c>
+      <c r="E222" s="2" t="s">
+        <v>598</v>
+      </c>
+      <c r="F222" s="2" t="s">
+        <v>601</v>
+      </c>
+      <c r="G222" s="2" t="s">
         <v>626</v>
-      </c>
-      <c r="D222" s="2" t="s">
-        <v>627</v>
-      </c>
-      <c r="E222" s="2" t="s">
-        <v>600</v>
-      </c>
-      <c r="F222" s="2" t="s">
-        <v>603</v>
-      </c>
-      <c r="G222" s="2" t="s">
-        <v>628</v>
       </c>
       <c r="H222" s="2" t="s">
         <v>21</v>
@@ -8513,22 +8530,22 @@
     </row>
     <row r="223" spans="1:8" ht="144.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A223" s="2" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="B223" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C223" s="3" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
       <c r="D223" s="2" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="E223" s="2" t="s">
         <v>19</v>
       </c>
       <c r="F223" s="2" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="G223" s="2" t="s">
         <v>17</v>
@@ -8539,13 +8556,13 @@
     </row>
     <row r="224" spans="1:8" ht="130.19999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A224" s="2" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="B224" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C224" s="3" t="s">
-        <v>630</v>
+        <v>628</v>
       </c>
       <c r="D224" s="2">
         <v>1</v>
@@ -8565,25 +8582,25 @@
     </row>
     <row r="225" spans="1:8" ht="144.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A225" s="2" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="B225" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C225" s="3" t="s">
+        <v>629</v>
+      </c>
+      <c r="D225" s="2" t="s">
+        <v>630</v>
+      </c>
+      <c r="E225" s="2" t="s">
+        <v>604</v>
+      </c>
+      <c r="F225" s="2" t="s">
         <v>631</v>
       </c>
-      <c r="D225" s="2" t="s">
+      <c r="G225" s="2" t="s">
         <v>632</v>
-      </c>
-      <c r="E225" s="2" t="s">
-        <v>606</v>
-      </c>
-      <c r="F225" s="2" t="s">
-        <v>633</v>
-      </c>
-      <c r="G225" s="2" t="s">
-        <v>634</v>
       </c>
       <c r="H225" s="2" t="s">
         <v>21</v>
@@ -8591,16 +8608,16 @@
     </row>
     <row r="226" spans="1:8" ht="130.19999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A226" s="2" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="B226" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C226" s="3" t="s">
-        <v>635</v>
+        <v>633</v>
       </c>
       <c r="D226" s="2" t="s">
-        <v>636</v>
+        <v>634</v>
       </c>
       <c r="E226" s="2" t="s">
         <v>298</v>
@@ -8617,25 +8634,25 @@
     </row>
     <row r="227" spans="1:8" ht="144.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A227" s="2" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="B227" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C227" s="3" t="s">
+        <v>635</v>
+      </c>
+      <c r="D227" s="2" t="s">
+        <v>636</v>
+      </c>
+      <c r="E227" s="2" t="s">
         <v>637</v>
-      </c>
-      <c r="D227" s="2" t="s">
-        <v>638</v>
-      </c>
-      <c r="E227" s="2" t="s">
-        <v>639</v>
       </c>
       <c r="F227" s="2" t="s">
         <v>278</v>
       </c>
       <c r="G227" s="2" t="s">
-        <v>640</v>
+        <v>638</v>
       </c>
       <c r="H227" s="2" t="s">
         <v>21</v>
@@ -8643,13 +8660,13 @@
     </row>
     <row r="228" spans="1:8" ht="115.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A228" s="2" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="B228" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C228" s="3" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
       <c r="D228" s="2">
         <v>2</v>
@@ -8669,25 +8686,25 @@
     </row>
     <row r="229" spans="1:8" ht="87" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A229" s="2" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="B229" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C229" s="3" t="s">
+        <v>640</v>
+      </c>
+      <c r="D229" s="2" t="s">
+        <v>641</v>
+      </c>
+      <c r="E229" s="2" t="s">
         <v>642</v>
       </c>
-      <c r="D229" s="2" t="s">
+      <c r="F229" s="2" t="s">
         <v>643</v>
       </c>
-      <c r="E229" s="2" t="s">
+      <c r="G229" s="2" t="s">
         <v>644</v>
-      </c>
-      <c r="F229" s="2" t="s">
-        <v>645</v>
-      </c>
-      <c r="G229" s="2" t="s">
-        <v>646</v>
       </c>
       <c r="H229" s="2" t="s">
         <v>21</v>
@@ -8695,25 +8712,25 @@
     </row>
     <row r="230" spans="1:8" ht="101.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A230" s="2" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="B230" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C230" s="3" t="s">
+        <v>645</v>
+      </c>
+      <c r="D230" s="2" t="s">
+        <v>646</v>
+      </c>
+      <c r="E230" s="2" t="s">
         <v>647</v>
       </c>
-      <c r="D230" s="2" t="s">
+      <c r="F230" s="2" t="s">
         <v>648</v>
       </c>
-      <c r="E230" s="2" t="s">
+      <c r="G230" s="2" t="s">
         <v>649</v>
-      </c>
-      <c r="F230" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="G230" s="2" t="s">
-        <v>651</v>
       </c>
       <c r="H230" s="2" t="s">
         <v>21</v>
@@ -8721,25 +8738,25 @@
     </row>
     <row r="231" spans="1:8" ht="115.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A231" s="2" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="B231" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C231" s="3" t="s">
+        <v>650</v>
+      </c>
+      <c r="D231" s="2" t="s">
+        <v>651</v>
+      </c>
+      <c r="E231" s="2" t="s">
         <v>652</v>
       </c>
-      <c r="D231" s="2" t="s">
+      <c r="F231" s="2" t="s">
         <v>653</v>
       </c>
-      <c r="E231" s="2" t="s">
+      <c r="G231" s="2" t="s">
         <v>654</v>
-      </c>
-      <c r="F231" s="2" t="s">
-        <v>655</v>
-      </c>
-      <c r="G231" s="2" t="s">
-        <v>656</v>
       </c>
       <c r="H231" s="2" t="s">
         <v>21</v>
@@ -8747,19 +8764,19 @@
     </row>
     <row r="232" spans="1:8" ht="159" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A232" s="2" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="B232" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C232" s="3" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="D232" s="2" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="E232" s="2" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="F232" s="2" t="s">
         <v>19</v>
@@ -8773,25 +8790,25 @@
     </row>
     <row r="233" spans="1:8" ht="101.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A233" s="2" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="B233" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C233" s="3" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="D233" s="2" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="E233" s="2" t="b">
         <v>0</v>
       </c>
       <c r="F233" s="2" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="G233" s="2" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="H233" s="2" t="s">
         <v>21</v>
@@ -8799,25 +8816,25 @@
     </row>
     <row r="234" spans="1:8" ht="144.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A234" s="2" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="B234" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C234" s="3" t="s">
-        <v>663</v>
+        <v>661</v>
       </c>
       <c r="D234" s="2" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="E234" s="2" t="s">
         <v>19</v>
       </c>
       <c r="F234" s="2" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="G234" s="2" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="H234" s="2" t="s">
         <v>21</v>
@@ -8825,25 +8842,25 @@
     </row>
     <row r="235" spans="1:8" ht="101.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A235" s="2" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="B235" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C235" s="3" t="s">
-        <v>664</v>
+        <v>662</v>
       </c>
       <c r="D235" s="2" t="s">
-        <v>665</v>
+        <v>663</v>
       </c>
       <c r="E235" s="2" t="s">
         <v>247</v>
       </c>
       <c r="F235" s="2" t="s">
-        <v>666</v>
+        <v>664</v>
       </c>
       <c r="G235" s="2" t="s">
-        <v>667</v>
+        <v>665</v>
       </c>
       <c r="H235" s="2" t="s">
         <v>21</v>
@@ -8851,25 +8868,25 @@
     </row>
     <row r="236" spans="1:8" ht="187.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A236" s="2" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="B236" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C236" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="D236" s="2" t="s">
+        <v>667</v>
+      </c>
+      <c r="E236" s="2" t="s">
         <v>668</v>
       </c>
-      <c r="D236" s="2" t="s">
+      <c r="F236" s="2" t="s">
         <v>669</v>
       </c>
-      <c r="E236" s="2" t="s">
+      <c r="G236" s="2" t="s">
         <v>670</v>
-      </c>
-      <c r="F236" s="2" t="s">
-        <v>671</v>
-      </c>
-      <c r="G236" s="2" t="s">
-        <v>672</v>
       </c>
       <c r="H236" s="2" t="s">
         <v>21</v>
@@ -8877,25 +8894,25 @@
     </row>
     <row r="237" spans="1:8" ht="159" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A237" s="2" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="B237" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C237" s="3" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="D237" s="2" t="s">
-        <v>638</v>
+        <v>636</v>
       </c>
       <c r="E237" s="2" t="s">
-        <v>674</v>
+        <v>672</v>
       </c>
       <c r="F237" s="2" t="s">
         <v>278</v>
       </c>
       <c r="G237" s="2" t="s">
-        <v>675</v>
+        <v>673</v>
       </c>
       <c r="H237" s="2" t="s">
         <v>21</v>
@@ -8903,25 +8920,25 @@
     </row>
     <row r="238" spans="1:8" ht="130.19999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A238" s="2" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="B238" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C238" s="3" t="s">
-        <v>676</v>
+        <v>674</v>
       </c>
       <c r="D238" s="2" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="E238" s="2" t="s">
         <v>298</v>
       </c>
       <c r="F238" s="2" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="G238" s="2" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="H238" s="2" t="s">
         <v>21</v>
@@ -8929,25 +8946,25 @@
     </row>
     <row r="239" spans="1:8" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A239" s="2" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="B239" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C239" s="3" t="s">
+        <v>675</v>
+      </c>
+      <c r="D239" s="2" t="s">
+        <v>676</v>
+      </c>
+      <c r="E239" s="2" t="s">
         <v>677</v>
       </c>
-      <c r="D239" s="2" t="s">
+      <c r="F239" s="2" t="s">
         <v>678</v>
       </c>
-      <c r="E239" s="2" t="s">
+      <c r="G239" s="2" t="s">
         <v>679</v>
-      </c>
-      <c r="F239" s="2" t="s">
-        <v>680</v>
-      </c>
-      <c r="G239" s="2" t="s">
-        <v>681</v>
       </c>
       <c r="H239" s="2" t="s">
         <v>21</v>
@@ -8955,13 +8972,13 @@
     </row>
     <row r="240" spans="1:8" ht="87" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A240" s="2" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="B240" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C240" s="3" t="s">
-        <v>682</v>
+        <v>680</v>
       </c>
       <c r="D240" s="2">
         <v>10</v>
@@ -8981,13 +8998,13 @@
     </row>
     <row r="241" spans="1:8" ht="130.19999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A241" s="2" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="B241" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C241" s="3" t="s">
-        <v>683</v>
+        <v>681</v>
       </c>
       <c r="D241" s="2" t="s">
         <v>298</v>
@@ -8996,7 +9013,7 @@
         <v>54</v>
       </c>
       <c r="F241" s="2" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="G241" s="2" t="s">
         <v>20</v>
@@ -9007,25 +9024,25 @@
     </row>
     <row r="242" spans="1:8" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A242" s="2" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="B242" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C242" s="3" t="s">
+        <v>683</v>
+      </c>
+      <c r="D242" s="2" t="s">
+        <v>684</v>
+      </c>
+      <c r="E242" s="2" t="s">
         <v>685</v>
       </c>
-      <c r="D242" s="2" t="s">
+      <c r="F242" s="2" t="s">
         <v>686</v>
       </c>
-      <c r="E242" s="2" t="s">
+      <c r="G242" s="2" t="s">
         <v>687</v>
-      </c>
-      <c r="F242" s="2" t="s">
-        <v>688</v>
-      </c>
-      <c r="G242" s="2" t="s">
-        <v>689</v>
       </c>
       <c r="H242" s="2" t="s">
         <v>21</v>
@@ -9033,25 +9050,25 @@
     </row>
     <row r="243" spans="1:8" ht="187.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A243" s="2" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="B243" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C243" s="3" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
       <c r="D243" s="2" t="s">
         <v>62</v>
       </c>
       <c r="E243" s="2" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
       <c r="F243" s="2" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="G243" s="2" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="H243" s="2" t="s">
         <v>29</v>
@@ -9059,25 +9076,25 @@
     </row>
     <row r="244" spans="1:8" ht="115.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A244" s="2" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="B244" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C244" s="3" t="s">
-        <v>693</v>
+        <v>691</v>
       </c>
       <c r="D244" s="2" t="s">
         <v>62</v>
       </c>
       <c r="E244" s="2" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
       <c r="F244" s="2" t="s">
+        <v>690</v>
+      </c>
+      <c r="G244" s="2" t="s">
         <v>692</v>
-      </c>
-      <c r="G244" s="2" t="s">
-        <v>694</v>
       </c>
       <c r="H244" s="2" t="s">
         <v>29</v>
@@ -9085,13 +9102,13 @@
     </row>
     <row r="245" spans="1:8" ht="173.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A245" s="2" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="B245" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C245" s="3" t="s">
-        <v>695</v>
+        <v>693</v>
       </c>
       <c r="D245" s="2">
         <v>3</v>
@@ -9111,22 +9128,22 @@
     </row>
     <row r="246" spans="1:8" ht="159" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A246" s="2" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="B246" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C246" s="3" t="s">
+        <v>694</v>
+      </c>
+      <c r="D246" s="2" t="s">
+        <v>695</v>
+      </c>
+      <c r="E246" s="2" t="s">
         <v>696</v>
       </c>
-      <c r="D246" s="2" t="s">
+      <c r="F246" s="2" t="s">
         <v>697</v>
-      </c>
-      <c r="E246" s="2" t="s">
-        <v>698</v>
-      </c>
-      <c r="F246" s="2" t="s">
-        <v>699</v>
       </c>
       <c r="G246" s="2" t="s">
         <v>149</v>
@@ -9137,25 +9154,25 @@
     </row>
     <row r="247" spans="1:8" ht="101.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A247" s="2" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="B247" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C247" s="3" t="s">
+        <v>698</v>
+      </c>
+      <c r="D247" s="2" t="s">
+        <v>699</v>
+      </c>
+      <c r="E247" s="2" t="s">
         <v>700</v>
       </c>
-      <c r="D247" s="2" t="s">
+      <c r="F247" s="2" t="s">
         <v>701</v>
       </c>
-      <c r="E247" s="2" t="s">
+      <c r="G247" s="2" t="s">
         <v>702</v>
-      </c>
-      <c r="F247" s="2" t="s">
-        <v>703</v>
-      </c>
-      <c r="G247" s="2" t="s">
-        <v>704</v>
       </c>
       <c r="H247" s="2" t="s">
         <v>21</v>
@@ -9163,22 +9180,22 @@
     </row>
     <row r="248" spans="1:8" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A248" s="2" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="B248" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C248" s="3" t="s">
+        <v>703</v>
+      </c>
+      <c r="D248" s="2" t="s">
+        <v>704</v>
+      </c>
+      <c r="E248" s="2" t="s">
         <v>705</v>
       </c>
-      <c r="D248" s="2" t="s">
+      <c r="F248" s="2" t="s">
         <v>706</v>
-      </c>
-      <c r="E248" s="2" t="s">
-        <v>707</v>
-      </c>
-      <c r="F248" s="2" t="s">
-        <v>708</v>
       </c>
       <c r="G248" s="2" t="s">
         <v>401</v>
@@ -9189,13 +9206,13 @@
     </row>
     <row r="249" spans="1:8" ht="87" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A249" s="2" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="B249" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C249" s="3" t="s">
-        <v>709</v>
+        <v>707</v>
       </c>
       <c r="D249" s="2">
         <v>0</v>
@@ -9204,7 +9221,7 @@
         <v>1</v>
       </c>
       <c r="F249" s="2" t="s">
-        <v>710</v>
+        <v>708</v>
       </c>
       <c r="G249" s="2" t="s">
         <v>245</v>
@@ -9215,13 +9232,13 @@
     </row>
     <row r="250" spans="1:8" ht="87" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A250" s="2" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="B250" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C250" s="3" t="s">
-        <v>711</v>
+        <v>709</v>
       </c>
       <c r="D250" s="2">
         <v>0</v>
@@ -9230,10 +9247,10 @@
         <v>1</v>
       </c>
       <c r="F250" s="2" t="s">
-        <v>712</v>
+        <v>710</v>
       </c>
       <c r="G250" s="2" t="s">
-        <v>710</v>
+        <v>708</v>
       </c>
       <c r="H250" s="2" t="s">
         <v>21</v>
@@ -9241,19 +9258,19 @@
     </row>
     <row r="251" spans="1:8" ht="115.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A251" s="2" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="B251" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C251" s="3" t="s">
+        <v>711</v>
+      </c>
+      <c r="D251" s="2" t="s">
+        <v>712</v>
+      </c>
+      <c r="E251" s="2" t="s">
         <v>713</v>
-      </c>
-      <c r="D251" s="2" t="s">
-        <v>714</v>
-      </c>
-      <c r="E251" s="2" t="s">
-        <v>715</v>
       </c>
       <c r="F251" s="2" t="s">
         <v>33</v>
@@ -9267,22 +9284,22 @@
     </row>
     <row r="252" spans="1:8" ht="115.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A252" s="2" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="B252" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C252" s="3" t="s">
-        <v>716</v>
+        <v>714</v>
       </c>
       <c r="D252" s="2" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
       <c r="E252" s="2" t="s">
         <v>62</v>
       </c>
       <c r="F252" s="2" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="G252" s="2" t="s">
         <v>17</v>
@@ -9293,25 +9310,25 @@
     </row>
     <row r="253" spans="1:8" ht="144.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A253" s="2" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="B253" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C253" s="3" t="s">
+        <v>715</v>
+      </c>
+      <c r="D253" s="2" t="s">
+        <v>716</v>
+      </c>
+      <c r="E253" s="2" t="s">
         <v>717</v>
       </c>
-      <c r="D253" s="2" t="s">
+      <c r="F253" s="2" t="s">
         <v>718</v>
       </c>
-      <c r="E253" s="2" t="s">
+      <c r="G253" s="2" t="s">
         <v>719</v>
-      </c>
-      <c r="F253" s="2" t="s">
-        <v>720</v>
-      </c>
-      <c r="G253" s="2" t="s">
-        <v>721</v>
       </c>
       <c r="H253" s="2" t="s">
         <v>21</v>
@@ -9319,13 +9336,13 @@
     </row>
     <row r="254" spans="1:8" ht="144.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A254" s="2" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="B254" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C254" s="3" t="s">
-        <v>722</v>
+        <v>720</v>
       </c>
       <c r="D254" s="2">
         <v>9</v>
@@ -9345,25 +9362,25 @@
     </row>
     <row r="255" spans="1:8" ht="159" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A255" s="2" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="B255" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C255" s="3" t="s">
-        <v>723</v>
+        <v>721</v>
       </c>
       <c r="D255" s="2" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="E255" s="2" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="F255" s="2" t="s">
         <v>155</v>
       </c>
       <c r="G255" s="2" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
       <c r="H255" s="2" t="s">
         <v>21</v>
@@ -9371,16 +9388,16 @@
     </row>
     <row r="256" spans="1:8" ht="144.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A256" s="2" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="B256" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C256" s="3" t="s">
-        <v>725</v>
+        <v>723</v>
       </c>
       <c r="D256" s="2" t="s">
-        <v>674</v>
+        <v>672</v>
       </c>
       <c r="E256" s="2" t="s">
         <v>278</v>
@@ -9389,7 +9406,7 @@
         <v>227</v>
       </c>
       <c r="G256" s="2" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="H256" s="2" t="s">
         <v>21</v>
@@ -9397,25 +9414,25 @@
     </row>
     <row r="257" spans="1:8" ht="101.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A257" s="2" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="B257" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C257" s="3" t="s">
-        <v>726</v>
+        <v>724</v>
       </c>
       <c r="D257" s="2" t="s">
         <v>62</v>
       </c>
       <c r="E257" s="2" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
       <c r="F257" s="2" t="s">
         <v>17</v>
       </c>
       <c r="G257" s="2" t="s">
-        <v>694</v>
+        <v>692</v>
       </c>
       <c r="H257" s="2" t="s">
         <v>23</v>
@@ -9423,25 +9440,25 @@
     </row>
     <row r="258" spans="1:8" ht="101.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A258" s="2" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="B258" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C258" s="3" t="s">
-        <v>727</v>
+        <v>725</v>
       </c>
       <c r="D258" s="2" t="s">
-        <v>638</v>
+        <v>636</v>
       </c>
       <c r="E258" s="2" t="s">
-        <v>728</v>
+        <v>726</v>
       </c>
       <c r="F258" s="2" t="s">
         <v>278</v>
       </c>
       <c r="G258" s="2" t="s">
-        <v>729</v>
+        <v>727</v>
       </c>
       <c r="H258" s="2" t="s">
         <v>21</v>
@@ -9449,25 +9466,25 @@
     </row>
     <row r="259" spans="1:8" ht="130.19999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A259" s="2" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="B259" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C259" s="3" t="s">
+        <v>728</v>
+      </c>
+      <c r="D259" s="2" t="s">
+        <v>690</v>
+      </c>
+      <c r="E259" s="2" t="s">
+        <v>446</v>
+      </c>
+      <c r="F259" s="2" t="s">
+        <v>729</v>
+      </c>
+      <c r="G259" s="2" t="s">
         <v>730</v>
-      </c>
-      <c r="D259" s="2" t="s">
-        <v>692</v>
-      </c>
-      <c r="E259" s="2" t="s">
-        <v>448</v>
-      </c>
-      <c r="F259" s="2" t="s">
-        <v>731</v>
-      </c>
-      <c r="G259" s="2" t="s">
-        <v>732</v>
       </c>
       <c r="H259" s="2" t="s">
         <v>21</v>
@@ -9475,25 +9492,25 @@
     </row>
     <row r="260" spans="1:8" ht="159" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A260" s="2" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="B260" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C260" s="3" t="s">
+        <v>731</v>
+      </c>
+      <c r="D260" s="2" t="s">
+        <v>732</v>
+      </c>
+      <c r="E260" s="2" t="s">
         <v>733</v>
       </c>
-      <c r="D260" s="2" t="s">
+      <c r="F260" s="2" t="s">
         <v>734</v>
       </c>
-      <c r="E260" s="2" t="s">
-        <v>735</v>
-      </c>
-      <c r="F260" s="2" t="s">
-        <v>736</v>
-      </c>
       <c r="G260" s="2" t="s">
-        <v>667</v>
+        <v>665</v>
       </c>
       <c r="H260" s="2" t="s">
         <v>21</v>
@@ -9501,25 +9518,25 @@
     </row>
     <row r="261" spans="1:8" ht="130.19999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A261" s="2" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="B261" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C261" s="3" t="s">
-        <v>737</v>
+        <v>735</v>
       </c>
       <c r="D261" s="2" t="s">
-        <v>738</v>
+        <v>736</v>
       </c>
       <c r="E261" s="2" t="s">
         <v>278</v>
       </c>
       <c r="F261" s="2" t="s">
-        <v>739</v>
+        <v>737</v>
       </c>
       <c r="G261" s="2" t="s">
-        <v>729</v>
+        <v>727</v>
       </c>
       <c r="H261" s="2" t="s">
         <v>23</v>
@@ -9527,25 +9544,25 @@
     </row>
     <row r="262" spans="1:8" ht="187.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A262" s="2" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="B262" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C262" s="3" t="s">
-        <v>740</v>
+        <v>738</v>
       </c>
       <c r="D262" s="2" t="s">
-        <v>741</v>
+        <v>739</v>
       </c>
       <c r="E262" s="2" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="F262" s="2" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="G262" s="2" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
       <c r="H262" s="2" t="s">
         <v>21</v>
@@ -9553,13 +9570,13 @@
     </row>
     <row r="263" spans="1:8" ht="144.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A263" s="2" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="B263" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C263" s="3" t="s">
-        <v>742</v>
+        <v>740</v>
       </c>
       <c r="D263" s="2">
         <v>15</v>
@@ -9579,25 +9596,25 @@
     </row>
     <row r="264" spans="1:8" ht="130.19999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A264" s="2" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="B264" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C264" s="3" t="s">
-        <v>743</v>
+        <v>741</v>
       </c>
       <c r="D264" s="2" t="s">
-        <v>744</v>
+        <v>742</v>
       </c>
       <c r="E264" s="2" t="s">
         <v>247</v>
       </c>
       <c r="F264" s="2" t="s">
-        <v>745</v>
+        <v>743</v>
       </c>
       <c r="G264" s="2" t="s">
-        <v>667</v>
+        <v>665</v>
       </c>
       <c r="H264" s="2" t="s">
         <v>21</v>
@@ -9605,25 +9622,25 @@
     </row>
     <row r="265" spans="1:8" ht="159" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A265" s="2" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="B265" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C265" s="3" t="s">
-        <v>746</v>
+        <v>744</v>
       </c>
       <c r="D265" s="2" t="s">
-        <v>747</v>
+        <v>745</v>
       </c>
       <c r="E265" s="2" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="F265" s="2" t="s">
-        <v>731</v>
+        <v>729</v>
       </c>
       <c r="G265" s="2" t="s">
-        <v>732</v>
+        <v>730</v>
       </c>
       <c r="H265" s="2" t="s">
         <v>21</v>
@@ -9631,25 +9648,25 @@
     </row>
     <row r="266" spans="1:8" ht="202.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A266" s="2" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="B266" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C266" s="3" t="s">
+        <v>746</v>
+      </c>
+      <c r="D266" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="E266" s="2" t="s">
+        <v>690</v>
+      </c>
+      <c r="F266" s="2" t="s">
+        <v>689</v>
+      </c>
+      <c r="G266" s="2" t="s">
         <v>748</v>
-      </c>
-      <c r="D266" s="2" t="s">
-        <v>749</v>
-      </c>
-      <c r="E266" s="2" t="s">
-        <v>692</v>
-      </c>
-      <c r="F266" s="2" t="s">
-        <v>691</v>
-      </c>
-      <c r="G266" s="2" t="s">
-        <v>750</v>
       </c>
       <c r="H266" s="2" t="s">
         <v>21</v>
@@ -9657,25 +9674,25 @@
     </row>
     <row r="267" spans="1:8" ht="115.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A267" s="2" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="B267" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C267" s="3" t="s">
-        <v>751</v>
+        <v>749</v>
       </c>
       <c r="D267" s="2" t="s">
-        <v>728</v>
+        <v>726</v>
       </c>
       <c r="E267" s="2" t="s">
-        <v>638</v>
+        <v>636</v>
       </c>
       <c r="F267" s="2" t="s">
-        <v>729</v>
+        <v>727</v>
       </c>
       <c r="G267" s="2" t="s">
-        <v>739</v>
+        <v>737</v>
       </c>
       <c r="H267" s="2" t="s">
         <v>21</v>
@@ -9683,13 +9700,13 @@
     </row>
     <row r="268" spans="1:8" ht="173.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A268" s="2" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="B268" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C268" s="3" t="s">
-        <v>752</v>
+        <v>750</v>
       </c>
       <c r="D268" s="2">
         <v>10</v>
@@ -9709,25 +9726,25 @@
     </row>
     <row r="269" spans="1:8" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A269" s="2" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="B269" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C269" s="3" t="s">
-        <v>753</v>
+        <v>751</v>
       </c>
       <c r="D269" s="2" t="s">
+        <v>676</v>
+      </c>
+      <c r="E269" s="2" t="s">
+        <v>677</v>
+      </c>
+      <c r="F269" s="2" t="s">
         <v>678</v>
       </c>
-      <c r="E269" s="2" t="s">
+      <c r="G269" s="2" t="s">
         <v>679</v>
-      </c>
-      <c r="F269" s="2" t="s">
-        <v>680</v>
-      </c>
-      <c r="G269" s="2" t="s">
-        <v>681</v>
       </c>
       <c r="H269" s="2" t="s">
         <v>21</v>
@@ -9735,25 +9752,25 @@
     </row>
     <row r="270" spans="1:8" ht="159" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A270" s="2" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="B270" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C270" s="3" t="s">
-        <v>754</v>
+        <v>752</v>
       </c>
       <c r="D270" s="2" t="s">
-        <v>750</v>
+        <v>748</v>
       </c>
       <c r="E270" s="2" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
       <c r="F270" s="2" t="s">
-        <v>755</v>
+        <v>753</v>
       </c>
       <c r="G270" s="2" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="H270" s="2" t="s">
         <v>21</v>
@@ -9761,13 +9778,13 @@
     </row>
     <row r="271" spans="1:8" ht="159" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A271" s="2" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="B271" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C271" s="3" t="s">
-        <v>756</v>
+        <v>754</v>
       </c>
       <c r="D271" s="2">
         <v>3</v>
@@ -9787,25 +9804,25 @@
     </row>
     <row r="272" spans="1:8" ht="130.19999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A272" s="2" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="B272" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C272" s="3" t="s">
+        <v>755</v>
+      </c>
+      <c r="D272" s="2" t="s">
+        <v>756</v>
+      </c>
+      <c r="E272" s="2" t="s">
         <v>757</v>
       </c>
-      <c r="D272" s="2" t="s">
+      <c r="F272" s="2" t="s">
         <v>758</v>
       </c>
-      <c r="E272" s="2" t="s">
+      <c r="G272" s="2" t="s">
         <v>759</v>
-      </c>
-      <c r="F272" s="2" t="s">
-        <v>760</v>
-      </c>
-      <c r="G272" s="2" t="s">
-        <v>761</v>
       </c>
       <c r="H272" s="2" t="s">
         <v>21</v>

</xml_diff>